<commit_message>
Strike the JBSS terminal value at the end of year 5
Year 6 free cash flow grows at 3.5% forever, so it is the first year of
the perpetuity and the terminal value belongs at the end of year 5. The
bridge now sums years 1 to 5 and divides year 6 cash flow by (WACC - g),
in the page and in the workbook's Bridge sheet alike. Enterprise value,
equity value and the 120.45 per share are unchanged -- the two framings
are the same quantity written two ways.

The forecast table also gains a grayed free cash flow growth line, which
is what makes the 3.5% from year 6 onward visible.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/jbss/jbss.xlsx
+++ b/docs/jbss/jbss.xlsx
@@ -1773,22 +1773,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PV of free cash flow, years 1 to 6</t>
+          <t>PV of free cash flow, years 1 to 5</t>
         </is>
       </c>
       <c r="B3" s="7">
-        <f>SUM(Model!B21:Model!G21)</f>
+        <f>SUM(Model!B21:Model!F21)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Terminal value at the end of year 6</t>
+          <t>Terminal value at the end of year 5</t>
         </is>
       </c>
       <c r="B4" s="7">
-        <f>Model!H19/(Inputs!$B$24-Inputs!$G$6)</f>
+        <f>Model!G19/(Inputs!$B$24-Inputs!$G$6)</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>B4/(1+Inputs!$B$24)^6</f>
+        <f>B4/(1+Inputs!$B$24)^5</f>
         <v/>
       </c>
     </row>
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="B26">
-        <f>IF(ABS(Bridge!B4-(1872544.2947459894))&gt;1e-06,"FAIL","ok")</f>
+        <f>IF(ABS(Bridge!B4-(1809221.5408173827))&gt;1e-06,"FAIL","ok")</f>
         <v/>
       </c>
     </row>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="B27">
-        <f>IF(ABS(Bridge!B5-(1180020.5395421663))&gt;1e-06,"FAIL","ok")</f>
+        <f>IF(ABS(Bridge!B5-(1231325.7803918268))&gt;1e-06,"FAIL","ok")</f>
         <v/>
       </c>
     </row>
@@ -10267,7 +10267,7 @@
         </is>
       </c>
       <c r="B28">
-        <f>IF(ABS(Bridge!B3-(337802.0659080064))&gt;1e-06,"FAIL","ok")</f>
+        <f>IF(ABS(Bridge!B3-(286496.8250583469))&gt;1e-06,"FAIL","ok")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Put the JBSS terminal value back on year 6
Striking it at the end of year 5 off year 6 cash flow is the same number
only when year 5's balance-sheet ratios are already the terminal ones,
as JBSS's are. Move one of them -- PP&E turnover or a working-capital
share -- and year 6 harvests the difference in a single year's cash
flow, which capitalised adds 18 to 40% to enterprise value. Year 6 as
the transition year counts that once, explicitly, which is the point of
it.

The grayed free cash flow growth line stays: terminal growth in the
year 7 cell is what says year 6 is a clean perpetuity base.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/jbss/jbss.xlsx
+++ b/docs/jbss/jbss.xlsx
@@ -1773,22 +1773,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PV of free cash flow, years 1 to 5</t>
+          <t>PV of free cash flow, years 1 to 6</t>
         </is>
       </c>
       <c r="B3" s="7">
-        <f>SUM(Model!B21:Model!F21)</f>
+        <f>SUM(Model!B21:Model!G21)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Terminal value at the end of year 5</t>
+          <t>Terminal value at the end of year 6</t>
         </is>
       </c>
       <c r="B4" s="7">
-        <f>Model!G19/(Inputs!$B$24-Inputs!$G$6)</f>
+        <f>Model!H19/(Inputs!$B$24-Inputs!$G$6)</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>B4/(1+Inputs!$B$24)^5</f>
+        <f>B4/(1+Inputs!$B$24)^6</f>
         <v/>
       </c>
     </row>
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="B26">
-        <f>IF(ABS(Bridge!B4-(1809221.5408173827))&gt;1e-06,"FAIL","ok")</f>
+        <f>IF(ABS(Bridge!B4-(1872544.2947459894))&gt;1e-06,"FAIL","ok")</f>
         <v/>
       </c>
     </row>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="B27">
-        <f>IF(ABS(Bridge!B5-(1231325.7803918268))&gt;1e-06,"FAIL","ok")</f>
+        <f>IF(ABS(Bridge!B5-(1180020.5395421663))&gt;1e-06,"FAIL","ok")</f>
         <v/>
       </c>
     </row>
@@ -10267,7 +10267,7 @@
         </is>
       </c>
       <c r="B28">
-        <f>IF(ABS(Bridge!B3-(286496.8250583469))&gt;1e-06,"FAIL","ok")</f>
+        <f>IF(ABS(Bridge!B3-(337802.0659080064))&gt;1e-06,"FAIL","ok")</f>
         <v/>
       </c>
     </row>

</xml_diff>